<commit_message>
Improve organic and social pack funnels
</commit_message>
<xml_diff>
--- a/content/member-assets/mobile-headlight-restoration/headlight-restoration-quote-calculator.xlsx
+++ b/content/member-assets/mobile-headlight-restoration/headlight-restoration-quote-calculator.xlsx
@@ -187,7 +187,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
           <t>What this is</t>
@@ -199,7 +199,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="54" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
           <t>Buyer</t>
@@ -259,7 +259,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
+    <row r="10" ht="54" customHeight="1">
       <c r="A10" t="inlineStr" s="6">
         <is>
           <t>How to use</t>
@@ -271,7 +271,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
+    <row r="11" ht="54" customHeight="1">
       <c r="A11" t="inlineStr" s="2">
         <is>
           <t>Delivery standards</t>
@@ -475,7 +475,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="54" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t>2. Draft</t>
@@ -497,7 +497,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
           <t>3. Flag</t>
@@ -519,7 +519,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="54" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
           <t>4. Approve</t>
@@ -541,7 +541,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="54" customHeight="1">
       <c r="A6" t="inlineStr" s="6">
         <is>
           <t>5. Deliver</t>
@@ -723,7 +723,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="54" customHeight="1">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -733,7 +733,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="54" customHeight="1">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -753,7 +753,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1436,7 +1436,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
           <t>Any cracks, moisture, previous restoration, or replacement history</t>
@@ -1762,7 +1762,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" t="inlineStr" s="6">
         <is>
           <t>Scope</t>
@@ -1774,7 +1774,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="72" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t>Boundary</t>
@@ -1786,7 +1786,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
           <t>Approval</t>
@@ -1798,7 +1798,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
           <t>Not included</t>

</xml_diff>